<commit_message>
Cleaned up display command outputs
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20251130.xlsx
+++ b/WorkBot/refactor-experimental/data/order_archive/DUTCH VALLEY FOOD DIST/DUTCH VALLEY FOOD DIST_Bakery_20251130.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,216 @@
         <v>59.37</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>832400</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Register Tape - Thermal (3.125" x 230')</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="E6" t="n">
+        <v>99.98</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>462225</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Joe Tea - Mango Lemonade</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>22.49</v>
+      </c>
+      <c r="E7" t="n">
+        <v>44.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>462180</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Joe Tea - Kiwi Strawberry</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>22.49</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22.49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>462105</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Joe Tea - Classic Lemonade</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>22.49</v>
+      </c>
+      <c r="E9" t="n">
+        <v>44.98</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>462175</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Joe Tea - Black Cherry</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>22.49</v>
+      </c>
+      <c r="E10" t="n">
+        <v>89.95999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>053387</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DV - Very Berry Pretzels</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>053125</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DV - Sour Neon Gummi Worms</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>053707</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DV - Gummi Sharks</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>27.77</v>
+      </c>
+      <c r="E13" t="n">
+        <v>27.77</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>053115</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DV - Gummi Bears (12 oz)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>33.98</v>
+      </c>
+      <c r="E14" t="n">
+        <v>33.98</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>616060</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DV - Chewey Caramel w/Pretzel (Sweet Jubilee)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>25.44</v>
+      </c>
+      <c r="E15" t="n">
+        <v>25.44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>